<commit_message>
Created the data provider utility for the Excel Data that is used in the CreateJobAPI
Added the LoginAPIJExcelDataDrivenTest and
CreateJobAPIExcelDataDrivenTest in testng-datadriven.xml file
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PhoenixTestData.xlsx
+++ b/src/test/resources/testData/PhoenixTestData.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTestData" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="CreateJobTestData" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="125725"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="57">
   <si>
     <t>username</t>
   </si>
@@ -31,19 +31,182 @@
   </si>
   <si>
     <t>iameng</t>
+  </si>
+  <si>
+    <t>mst_service_location_id</t>
+  </si>
+  <si>
+    <t>mst_platform_id</t>
+  </si>
+  <si>
+    <t>mst_warrenty_status_id</t>
+  </si>
+  <si>
+    <t>mst_oem_id</t>
+  </si>
+  <si>
+    <t>customer__first_name</t>
+  </si>
+  <si>
+    <t>customer__last_name</t>
+  </si>
+  <si>
+    <t>customer__mobile_number</t>
+  </si>
+  <si>
+    <t>customer__mobile_number_alt</t>
+  </si>
+  <si>
+    <t>customer__email_id</t>
+  </si>
+  <si>
+    <t>customer__email_id_alt</t>
+  </si>
+  <si>
+    <t>customer_address__flat_number</t>
+  </si>
+  <si>
+    <t>customer_address__apartment_name</t>
+  </si>
+  <si>
+    <t>customer_address__street_name</t>
+  </si>
+  <si>
+    <t>customer_address__landmark</t>
+  </si>
+  <si>
+    <t>customer_address__area</t>
+  </si>
+  <si>
+    <t>customer_address__pincode</t>
+  </si>
+  <si>
+    <t>customer_address__country</t>
+  </si>
+  <si>
+    <t>customer_address__state</t>
+  </si>
+  <si>
+    <t>customer_product__dop</t>
+  </si>
+  <si>
+    <t>customer_product__serial_number</t>
+  </si>
+  <si>
+    <t>customer_product__imei1</t>
+  </si>
+  <si>
+    <t>customer_product__imei2</t>
+  </si>
+  <si>
+    <t>customer_product__popurl</t>
+  </si>
+  <si>
+    <t>customer_product__product_id</t>
+  </si>
+  <si>
+    <t>customer_product__mst_model_id</t>
+  </si>
+  <si>
+    <t>problems__id</t>
+  </si>
+  <si>
+    <t>problems__remark</t>
+  </si>
+  <si>
+    <t>Rasheed</t>
+  </si>
+  <si>
+    <t>Bergstrom</t>
+  </si>
+  <si>
+    <t>785-682-6718</t>
+  </si>
+  <si>
+    <t>Arnaldo_Boehm99@yahoo.com</t>
+  </si>
+  <si>
+    <t>20B</t>
+  </si>
+  <si>
+    <t>Atria</t>
+  </si>
+  <si>
+    <t>HMTMain</t>
+  </si>
+  <si>
+    <t>HMT</t>
+  </si>
+  <si>
+    <t>Jalahalli</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Karnataka</t>
+  </si>
+  <si>
+    <t>2025-04-07T18:30:00.000Z</t>
+  </si>
+  <si>
+    <t>Battery issue</t>
+  </si>
+  <si>
+    <t>Manasi</t>
+  </si>
+  <si>
+    <t>Ayansh</t>
+  </si>
+  <si>
+    <t>Anushree</t>
+  </si>
+  <si>
+    <t>95362420558678</t>
+  </si>
+  <si>
+    <t>96362420558890</t>
+  </si>
+  <si>
+    <t>97362420558589</t>
+  </si>
+  <si>
+    <t>98362420558895</t>
+  </si>
+  <si>
+    <t>785-682-6719</t>
+  </si>
+  <si>
+    <t>785-682-6720</t>
+  </si>
+  <si>
+    <t>785-682-6721</t>
+  </si>
+  <si>
+    <t>785-682-6722</t>
+  </si>
+  <si>
+    <t>Arnaldo_Boehm98@yahoo.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -63,13 +226,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -404,9 +574,459 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="37.109375" customWidth="1"/>
+    <col min="11" max="11" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.21875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O1" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>21</v>
+      </c>
+      <c r="R1" t="s">
+        <v>22</v>
+      </c>
+      <c r="S1" t="s">
+        <v>23</v>
+      </c>
+      <c r="T1" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" t="s">
+        <v>25</v>
+      </c>
+      <c r="V1" t="s">
+        <v>26</v>
+      </c>
+      <c r="W1" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="K2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P2">
+        <v>560089</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>41</v>
+      </c>
+      <c r="R2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S2" t="s">
+        <v>43</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="W2" t="s">
+        <v>43</v>
+      </c>
+      <c r="X2">
+        <v>1</v>
+      </c>
+      <c r="Y2">
+        <v>1</v>
+      </c>
+      <c r="Z2">
+        <v>1</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27">
+      <c r="A3">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="K3" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P3">
+        <v>560089</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>41</v>
+      </c>
+      <c r="R3" t="s">
+        <v>42</v>
+      </c>
+      <c r="S3" t="s">
+        <v>43</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="W3" t="s">
+        <v>43</v>
+      </c>
+      <c r="X3">
+        <v>1</v>
+      </c>
+      <c r="Y3">
+        <v>1</v>
+      </c>
+      <c r="Z3">
+        <v>1</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="K4" t="s">
+        <v>36</v>
+      </c>
+      <c r="L4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" t="s">
+        <v>39</v>
+      </c>
+      <c r="O4" t="s">
+        <v>40</v>
+      </c>
+      <c r="P4">
+        <v>560089</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>41</v>
+      </c>
+      <c r="R4" t="s">
+        <v>42</v>
+      </c>
+      <c r="S4" t="s">
+        <v>43</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="W4" t="s">
+        <v>43</v>
+      </c>
+      <c r="X4">
+        <v>1</v>
+      </c>
+      <c r="Y4">
+        <v>1</v>
+      </c>
+      <c r="Z4">
+        <v>1</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27">
+      <c r="A5">
+        <v>0</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L5" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O5" t="s">
+        <v>40</v>
+      </c>
+      <c r="P5">
+        <v>560089</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>41</v>
+      </c>
+      <c r="R5" t="s">
+        <v>42</v>
+      </c>
+      <c r="S5" t="s">
+        <v>43</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="W5" t="s">
+        <v>43</v>
+      </c>
+      <c r="X5">
+        <v>1</v>
+      </c>
+      <c r="Y5">
+        <v>1</v>
+      </c>
+      <c r="Z5">
+        <v>1</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J2" r:id="rId1"/>
+    <hyperlink ref="J3" r:id="rId2"/>
+    <hyperlink ref="J4" r:id="rId3"/>
+    <hyperlink ref="J5" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>